<commit_message>
Todo Valle en 98,9 h y el modo oscuro vuelve a pintar el plan
Con 60 minutos de busqueda el plan de 90 sedes en cuatro cuadrillas baja de
100,1 h a 98,9 h, mismo territorio.

Al pasar a oscuro el mapa quedaba sin escuelas ni cuadrillas, en el Valle y en
Risaralda. Las capas se repintaban en styledata, que salta antes de que llegue
el estilo nuevo; ahora se repintan en style.load.
</commit_message>
<xml_diff>
--- a/public/datos/plan_cuadrillas_todas_4_cuadrillas.xlsx
+++ b/public/datos/plan_cuadrillas_todas_4_cuadrillas.xlsx
@@ -3247,17 +3247,17 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SAN JUAN BOSCO</t>
+          <t>POLICARPA SALAVARRIETA</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA SAN JUAN BOSCO</t>
+          <t>INSTITUCION EDUCATIVA ALFONSO ZAWADZKY</t>
         </is>
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>276890000237</t>
+          <t>176890000020</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -3267,12 +3267,12 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>VEREDA SAN JUAN</t>
+          <t>KR 6 6 67</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -3286,20 +3286,20 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>59.23</v>
+        <v>0.73</v>
       </c>
       <c r="Q22" t="n">
-        <v>63.8</v>
+        <v>0.37</v>
       </c>
       <c r="R22" t="n">
-        <v>123</v>
+        <v>3.1</v>
       </c>
       <c r="S22" t="n">
-        <v>46.8</v>
+        <v>0.8</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>No habitable</t>
+          <t>Peligro de colapso</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -3309,32 +3309,32 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>camino destapado</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="Z22" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 23 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 10 m de esa vía.</t>
         </is>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>MEDIACANOA - MIRAVALLE - CAMPO ALEGRE - CRUCE VIA 2302</t>
+          <t>Carrera 6</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -3343,10 +3343,10 @@
         </is>
       </c>
       <c r="AC22" t="n">
-        <v>3.962278</v>
+        <v>3.85991597259148</v>
       </c>
       <c r="AD22" t="n">
-        <v>-76.40526699999999</v>
+        <v>-76.38388046730552</v>
       </c>
     </row>
     <row r="23">
@@ -3365,14 +3365,14 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>martes</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -3381,7 +3381,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>POLICARPA SALAVARRIETA</t>
+          <t>ALFONSO ZAWADZKY</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -3391,7 +3391,7 @@
       </c>
       <c r="J23" s="3" t="inlineStr">
         <is>
-          <t>176890000020</t>
+          <t>176890000305</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -3406,7 +3406,7 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>KR 6 6 67</t>
+          <t>KR 5 5 79</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -3416,24 +3416,24 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>Buga</t>
+          <t>Yotoco</t>
         </is>
       </c>
       <c r="P23" t="n">
-        <v>0.73</v>
+        <v>0.37</v>
       </c>
       <c r="Q23" t="n">
-        <v>22.81</v>
+        <v>1.99</v>
       </c>
       <c r="R23" t="n">
-        <v>25.8</v>
+        <v>3.1</v>
       </c>
       <c r="S23" t="n">
-        <v>14.1</v>
+        <v>0.8</v>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>Peligro de colapso</t>
+          <t>No habitable</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -3443,32 +3443,32 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Riesgo inminente de colapso</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X23" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>camino rural sin categoria</t>
         </is>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="Z23" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 10 m de esa vía.</t>
+          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 15 m de esa vía.</t>
         </is>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>Carrera 6</t>
+          <t>Calle 6</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -3477,10 +3477,10 @@
         </is>
       </c>
       <c r="AC23" t="n">
-        <v>3.85991597259148</v>
+        <v>3.86056963997</v>
       </c>
       <c r="AD23" t="n">
-        <v>-76.38388046730552</v>
+        <v>-76.38430955440001</v>
       </c>
     </row>
     <row r="24">
@@ -3506,88 +3506,103 @@
         <v>3</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>BID (43)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>SAN JUAN BOSCO</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>INSTITUCION EDUCATIVA SAN JUAN BOSCO</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>276890000237</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>YOTOCO</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>VEREDA SAN JUAN</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Yotoco</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
           <t>Buga</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>NARCISO CABAL SALCEDO - SEDE PRINCIPAL</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA NARCISO CABAL SALCEDO</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>176111000469</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Buga</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>Urbana</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>CL 2 8 47</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Yotoco</t>
-        </is>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>Buga</t>
-        </is>
-      </c>
       <c r="P24" t="n">
-        <v>22.81</v>
+        <v>59.23</v>
       </c>
       <c r="Q24" t="n">
-        <v>2.28</v>
+        <v>75.05</v>
       </c>
       <c r="R24" t="n">
-        <v>25.8</v>
+        <v>134.3</v>
       </c>
       <c r="S24" t="n">
-        <v>14.1</v>
+        <v>51.6</v>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>No habitable</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>aprobado por la mesa</t>
+        </is>
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X24" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>camino destapado</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 15 m de esa vía.</t>
+          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 23 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>MEDIACANOA - MIRAVALLE - CAMPO ALEGRE - CRUCE VIA 2302</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -3596,10 +3611,10 @@
         </is>
       </c>
       <c r="AC24" t="n">
-        <v>3.894397016</v>
+        <v>3.962278</v>
       </c>
       <c r="AD24" t="n">
-        <v>-76.29777</v>
+        <v>-76.40526699999999</v>
       </c>
     </row>
     <row r="25">
@@ -3634,17 +3649,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>CRISTOBAL COLÓN</t>
+          <t>ESC JOAQUIN CAMILO TORRES</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA MANUEL ANTONIO SANCLEMENTE</t>
+          <t>INSTITUCION EDUCATIVA TULIO ENRIQUE TASCON</t>
         </is>
       </c>
       <c r="J25" s="3" t="inlineStr">
         <is>
-          <t>276111001087</t>
+          <t>176111001171</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3659,7 +3674,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>VDA GUADUALEJO</t>
+          <t>CL 15 9 45</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3673,20 +3688,20 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>4.38</v>
+        <v>4.08</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.54</v>
+        <v>4.46</v>
       </c>
       <c r="R25" t="n">
-        <v>9.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="S25" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Riesgo inminente de colapso</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
@@ -3706,12 +3721,7 @@
       </c>
       <c r="Z25" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 8 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>Calle 4A</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 12 m de esa vía.</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -3720,10 +3730,10 @@
         </is>
       </c>
       <c r="AC25" t="n">
-        <v>3.893611111</v>
+        <v>3.9055</v>
       </c>
       <c r="AD25" t="n">
-        <v>-76.29111</v>
+        <v>-76.29489</v>
       </c>
     </row>
     <row r="26">
@@ -3758,17 +3768,17 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>MANUEL ANTONIO SANCLEMENTE - SEDE PRINCIPAL</t>
+          <t>EL PLACER - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA MANUEL ANTONIO SANCLEMENTE</t>
+          <t>INSTITUCION EDUCATIVA EL PLACER</t>
         </is>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>176111000515</t>
+          <t>276111000102</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -3778,12 +3788,12 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>CL 4 A 1 E 26</t>
+          <t>CORREG EL PLACER</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3797,16 +3807,16 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>0.54</v>
+        <v>4.46</v>
       </c>
       <c r="Q26" t="n">
-        <v>4.14</v>
+        <v>1.2</v>
       </c>
       <c r="R26" t="n">
-        <v>9.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="S26" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="V26" t="inlineStr">
         <is>
@@ -3820,7 +3830,7 @@
       </c>
       <c r="X26" t="inlineStr">
         <is>
-          <t>via terciaria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y26" t="inlineStr">
@@ -3830,12 +3840,12 @@
       </c>
       <c r="Z26" t="inlineStr">
         <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 30 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 30 m de esa vía.</t>
         </is>
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>Calle 4</t>
+          <t>Calle 6</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3844,10 +3854,10 @@
         </is>
       </c>
       <c r="AC26" t="n">
-        <v>3.89307</v>
+        <v>3.898611</v>
       </c>
       <c r="AD26" t="n">
-        <v>-76.29131</v>
+        <v>-76.30056</v>
       </c>
     </row>
     <row r="27">
@@ -3882,17 +3892,17 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>ESC JOAQUIN CAMILO TORRES</t>
+          <t>ACADEMICO - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA TULIO ENRIQUE TASCON</t>
+          <t>INSTITUCION EDUCATIVA ACADEMICO</t>
         </is>
       </c>
       <c r="J27" s="3" t="inlineStr">
         <is>
-          <t>176111001171</t>
+          <t>176111001104</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -3907,7 +3917,7 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>CL 15 9 45</t>
+          <t>KR 9 A 2 55 SUR</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -3917,29 +3927,29 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>Caicedonia</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="P27" t="n">
-        <v>4.08</v>
+        <v>3.44</v>
       </c>
       <c r="Q27" t="n">
-        <v>1.59</v>
+        <v>1.17</v>
       </c>
       <c r="R27" t="n">
-        <v>106</v>
+        <v>6.9</v>
       </c>
       <c r="S27" t="n">
-        <v>98.7</v>
+        <v>2</v>
       </c>
       <c r="V27" t="inlineStr">
         <is>
-          <t>Riesgo inminente de colapso</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W27" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X27" t="inlineStr">
@@ -3954,7 +3964,12 @@
       </c>
       <c r="Z27" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 12 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 25 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>Carrera 9</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3963,10 +3978,10 @@
         </is>
       </c>
       <c r="AC27" t="n">
-        <v>3.9055</v>
+        <v>3.892781656</v>
       </c>
       <c r="AD27" t="n">
-        <v>-76.29489</v>
+        <v>-76.29845</v>
       </c>
     </row>
     <row r="28">
@@ -4001,17 +4016,17 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>ESC JORGE ELIECER GAITAN</t>
+          <t>NARCISO CABAL SALCEDO - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA TULIO ENRIQUE TASCON</t>
+          <t>INSTITUCION EDUCATIVA NARCISO CABAL SALCEDO</t>
         </is>
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>176111001139</t>
+          <t>176111000469</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -4026,7 +4041,7 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>CR 10 NO 18-81</t>
+          <t>CL 2 8 47</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -4036,29 +4051,29 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>Caicedonia</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="P28" t="n">
-        <v>1.59</v>
+        <v>1.17</v>
       </c>
       <c r="Q28" t="n">
-        <v>100.29</v>
+        <v>2.28</v>
       </c>
       <c r="R28" t="n">
-        <v>106</v>
+        <v>6.9</v>
       </c>
       <c r="S28" t="n">
-        <v>98.7</v>
+        <v>2</v>
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>Riesgo inminente de colapso</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X28" t="inlineStr">
@@ -4073,12 +4088,7 @@
       </c>
       <c r="Z28" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 29 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA28" t="inlineStr">
-        <is>
-          <t>Carrera 10</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 15 m de esa vía.</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -4087,10 +4097,10 @@
         </is>
       </c>
       <c r="AC28" t="n">
-        <v>3.90894</v>
+        <v>3.894397016</v>
       </c>
       <c r="AD28" t="n">
-        <v>-76.29465</v>
+        <v>-76.29777</v>
       </c>
     </row>
     <row r="29">
@@ -4120,27 +4130,27 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>BOLIVARIANO</t>
+          <t>ESC JORGE ELIECER GAITAN</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA BOLIVARIANO</t>
+          <t>INSTITUCION EDUCATIVA TULIO ENRIQUE TASCON</t>
         </is>
       </c>
       <c r="J29" s="3" t="inlineStr">
         <is>
-          <t>176122000380</t>
+          <t>176111001139</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>CAICEDONIA</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -4150,44 +4160,34 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>CL 5 11 15</t>
+          <t>CR 10 NO 18-81</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Caicedonia</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>Andalucia</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="P29" t="n">
-        <v>1.47</v>
+        <v>3.97</v>
       </c>
       <c r="Q29" t="n">
-        <v>59.43</v>
+        <v>3.43</v>
       </c>
       <c r="R29" t="n">
-        <v>92.90000000000001</v>
+        <v>16.9</v>
       </c>
       <c r="S29" t="n">
-        <v>79.7</v>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>Peligro de colapso</t>
-        </is>
-      </c>
-      <c r="U29" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
+        <v>4.5</v>
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Riesgo inminente de colapso</t>
         </is>
       </c>
       <c r="W29" t="inlineStr">
@@ -4207,12 +4207,12 @@
       </c>
       <c r="Z29" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 15 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 29 m de esa vía.</t>
         </is>
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t>Calle 5</t>
+          <t>Carrera 10</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -4221,10 +4221,10 @@
         </is>
       </c>
       <c r="AC29" t="n">
-        <v>4.329633623</v>
+        <v>3.90894</v>
       </c>
       <c r="AD29" t="n">
-        <v>-75.82531724</v>
+        <v>-76.29465</v>
       </c>
     </row>
     <row r="30">
@@ -4254,27 +4254,27 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>SANTA CECILIA</t>
+          <t>INSTITUTO TECNICO AGRICOLA-SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA EFRAIN VARELA VACA</t>
+          <t>INSTITUCION EDUCATIVA AGRICOLA DE GUADALAJARA DE BUGA</t>
         </is>
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>176895000231</t>
+          <t>176111000507</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>ZARZAL</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -4284,54 +4284,44 @@
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>CL 10 KR 10 EQ</t>
+          <t>CL 23 KR 9 A</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Caicedonia</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>Andalucia</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="P30" t="n">
-        <v>59.43</v>
+        <v>3.43</v>
       </c>
       <c r="Q30" t="n">
-        <v>31.96</v>
+        <v>9.52</v>
       </c>
       <c r="R30" t="n">
-        <v>92.90000000000001</v>
+        <v>16.9</v>
       </c>
       <c r="S30" t="n">
-        <v>79.7</v>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>Peligro de colapso</t>
-        </is>
-      </c>
-      <c r="U30" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
+        <v>4.5</v>
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>Riesgo inminente de colapso</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W30" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X30" t="inlineStr">
         <is>
-          <t>via terciaria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr">
@@ -4341,12 +4331,7 @@
       </c>
       <c r="Z30" t="inlineStr">
         <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 18 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA30" t="inlineStr">
-        <is>
-          <t>Carrera 10</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 32 m de esa vía.</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -4355,10 +4340,10 @@
         </is>
       </c>
       <c r="AC30" t="n">
-        <v>4.3959229</v>
+        <v>3.914166667</v>
       </c>
       <c r="AD30" t="n">
-        <v>-76.0708454</v>
+        <v>-76.2925</v>
       </c>
     </row>
     <row r="31">
@@ -4393,17 +4378,17 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>TULIO ENRIQUE TASCON CHAMBIMBAL - SEDE PRINCIPAL</t>
+          <t>CRISTOBAL COLÓN</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA TULIO ENRIQUE TASCON CHAMBIMBAL</t>
+          <t>INSTITUCION EDUCATIVA MANUEL ANTONIO SANCLEMENTE</t>
         </is>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>276111000781</t>
+          <t>276111001087</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -4413,17 +4398,17 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>CHAMBIMBAL</t>
+          <t>VDA GUADUALEJO</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Andalucia</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -4432,40 +4417,45 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>41.77</v>
+        <v>4.38</v>
       </c>
       <c r="Q31" t="n">
-        <v>16.89</v>
+        <v>0.54</v>
       </c>
       <c r="R31" t="n">
-        <v>66.8</v>
+        <v>9.1</v>
       </c>
       <c r="S31" t="n">
-        <v>46.6</v>
+        <v>2.8</v>
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X31" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 187 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 8 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>Calle 4A</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
@@ -4474,10 +4464,10 @@
         </is>
       </c>
       <c r="AC31" t="n">
-        <v>3.956111</v>
+        <v>3.893611111</v>
       </c>
       <c r="AD31" t="n">
-        <v>-76.30028</v>
+        <v>-76.29111</v>
       </c>
     </row>
     <row r="32">
@@ -4512,17 +4502,17 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>GUADALAJARA</t>
+          <t>MANUEL ANTONIO SANCLEMENTE - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA GRAN COLOMBIA</t>
+          <t>INSTITUCION EDUCATIVA MANUEL ANTONIO SANCLEMENTE</t>
         </is>
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>176111000604</t>
+          <t>176111000515</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -4537,12 +4527,12 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>CR 27 NO 14-23</t>
+          <t>CL 4 A 1 E 26</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Andalucia</t>
+          <t>Buga</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -4551,30 +4541,30 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>16.89</v>
+        <v>0.54</v>
       </c>
       <c r="Q32" t="n">
-        <v>8.17</v>
+        <v>4.14</v>
       </c>
       <c r="R32" t="n">
-        <v>66.8</v>
+        <v>9.1</v>
       </c>
       <c r="S32" t="n">
-        <v>46.6</v>
+        <v>2.8</v>
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>Riesgo inminente de colapso</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X32" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="Y32" t="inlineStr">
@@ -4584,12 +4574,12 @@
       </c>
       <c r="Z32" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 22 m de esa vía.</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 30 m de esa vía.</t>
         </is>
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>Carrera 27</t>
+          <t>Calle 4</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
@@ -4598,10 +4588,10 @@
         </is>
       </c>
       <c r="AC32" t="n">
-        <v>3.911822</v>
+        <v>3.89307</v>
       </c>
       <c r="AD32" t="n">
-        <v>-76.30735</v>
+        <v>-76.29131</v>
       </c>
     </row>
     <row r="33">
@@ -4636,17 +4626,17 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>INSTITUTO TECNICO AGRICOLA-SEDE PRINCIPAL</t>
+          <t>GUADALAJARA</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA AGRICOLA DE GUADALAJARA DE BUGA</t>
+          <t>INSTITUCION EDUCATIVA GRAN COLOMBIA</t>
         </is>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>176111000507</t>
+          <t>176111000604</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -4661,7 +4651,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>CL 23 KR 9 A</t>
+          <t>CR 27 NO 14-23</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -4671,29 +4661,29 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>Andalucia</t>
+          <t>Caicedonia</t>
         </is>
       </c>
       <c r="P33" t="n">
-        <v>7.33</v>
+        <v>7.65</v>
       </c>
       <c r="Q33" t="n">
-        <v>35.55</v>
+        <v>34.79</v>
       </c>
       <c r="R33" t="n">
-        <v>45.9</v>
+        <v>111.8</v>
       </c>
       <c r="S33" t="n">
-        <v>38.3</v>
+        <v>102.8</v>
       </c>
       <c r="V33" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Riesgo inminente de colapso</t>
         </is>
       </c>
       <c r="W33" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X33" t="inlineStr">
@@ -4708,7 +4698,12 @@
       </c>
       <c r="Z33" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 32 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 22 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AA33" t="inlineStr">
+        <is>
+          <t>Carrera 27</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
@@ -4717,10 +4712,10 @@
         </is>
       </c>
       <c r="AC33" t="n">
-        <v>3.914166667</v>
+        <v>3.911822</v>
       </c>
       <c r="AD33" t="n">
-        <v>-76.2925</v>
+        <v>-76.30735</v>
       </c>
     </row>
     <row r="34">
@@ -4790,20 +4785,20 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>Andalucia</t>
+          <t>Caicedonia</t>
         </is>
       </c>
       <c r="P34" t="n">
-        <v>35.55</v>
+        <v>34.79</v>
       </c>
       <c r="Q34" t="n">
-        <v>2.99</v>
+        <v>69.31</v>
       </c>
       <c r="R34" t="n">
-        <v>45.9</v>
+        <v>111.8</v>
       </c>
       <c r="S34" t="n">
-        <v>38.3</v>
+        <v>102.8</v>
       </c>
       <c r="T34" t="inlineStr">
         <is>
@@ -4889,22 +4884,22 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>NUESTRA SEÑORA DE CHIQUINQUIRA</t>
+          <t>BOLIVARIANO</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DE CHIQUINQUIRA</t>
+          <t>INSTITUCION EDUCATIVA BOLIVARIANO</t>
         </is>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
-          <t>176622000076</t>
+          <t>176122000380</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>ROLDANILLO</t>
+          <t>CAICEDONIA</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -4914,34 +4909,34 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>CL 4 5 38</t>
+          <t>CL 5 11 15</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
+          <t>Caicedonia</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
           <t>Andalucia</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>Tulua</t>
-        </is>
-      </c>
       <c r="P35" t="n">
-        <v>48.65</v>
+        <v>1.47</v>
       </c>
       <c r="Q35" t="n">
-        <v>14.74</v>
+        <v>59.43</v>
       </c>
       <c r="R35" t="n">
-        <v>114.3</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="S35" t="n">
-        <v>93.2</v>
+        <v>79.7</v>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>Uso restringido</t>
+          <t>Peligro de colapso</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4951,12 +4946,12 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X35" t="inlineStr">
@@ -4971,12 +4966,12 @@
       </c>
       <c r="Z35" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 10 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 15 m de esa vía.</t>
         </is>
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t>Carrera 5</t>
+          <t>Calle 5</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4985,10 +4980,10 @@
         </is>
       </c>
       <c r="AC35" t="n">
-        <v>4.412260842287796</v>
+        <v>4.329633623</v>
       </c>
       <c r="AD35" t="n">
-        <v>-76.15737540436542</v>
+        <v>-75.82531724</v>
       </c>
     </row>
     <row r="36">
@@ -5023,22 +5018,22 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>MANUEL DOLORES MONDRAGON</t>
+          <t>SANTA CECILIA</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA MANUEL DOLORES MONDRAGON</t>
+          <t>INSTITUCION EDUCATIVA EFRAIN VARELA VACA</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>176100000254</t>
+          <t>176895000231</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>BOLIVAR</t>
+          <t>ZARZAL</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -5048,34 +5043,34 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>KR 2 2 66</t>
+          <t>CL 10 KR 10 EQ</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
+          <t>Caicedonia</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
           <t>Andalucia</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>Tulua</t>
-        </is>
-      </c>
       <c r="P36" t="n">
-        <v>14.74</v>
+        <v>59.43</v>
       </c>
       <c r="Q36" t="n">
-        <v>50.86</v>
+        <v>31.96</v>
       </c>
       <c r="R36" t="n">
-        <v>114.3</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="S36" t="n">
-        <v>93.2</v>
+        <v>79.7</v>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>Uso restringido</t>
+          <t>Peligro de colapso</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -5085,17 +5080,17 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Riesgo inminente de colapso</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X36" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="Y36" t="inlineStr">
@@ -5105,12 +5100,12 @@
       </c>
       <c r="Z36" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 43 m de esa vía.</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 18 m de esa vía.</t>
         </is>
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>BOLIVAR CRUCE CON VIA DE INVIAS 2302 EN TRAMO 23020 INICIO A 52m DE INICIO DE VIA 10023VL02B</t>
+          <t>Carrera 10</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -5119,10 +5114,10 @@
         </is>
       </c>
       <c r="AC36" t="n">
-        <v>4.340805</v>
+        <v>4.3959229</v>
       </c>
       <c r="AD36" t="n">
-        <v>-76.17979800000001</v>
+        <v>-76.0708454</v>
       </c>
     </row>
     <row r="37">
@@ -5152,27 +5147,27 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Tuluá</t>
+          <t>BID (43)</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>SEDE PRINCIPAL LICEO MODERNO</t>
+          <t>NUESTRA SEÑORA DE CHIQUINQUIRA</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA MODERNA DE TULUA</t>
+          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DE CHIQUINQUIRA</t>
         </is>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>176834000106</t>
+          <t>176622000076</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Tuluá</t>
+          <t>ROLDANILLO</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
@@ -5182,44 +5177,54 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>IND CALLE 27 NO. 6AW 240</t>
+          <t>CL 4 5 38</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
+          <t>Andalucia</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
           <t>Tulua</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>Tulua</t>
-        </is>
-      </c>
       <c r="P37" t="n">
-        <v>7.41</v>
+        <v>48.65</v>
       </c>
       <c r="Q37" t="n">
-        <v>42.09</v>
+        <v>14.74</v>
       </c>
       <c r="R37" t="n">
-        <v>100.2</v>
+        <v>114.3</v>
       </c>
       <c r="S37" t="n">
-        <v>57</v>
+        <v>93.2</v>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>Uso restringido</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>aprobado por la mesa</t>
+        </is>
       </c>
       <c r="V37" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X37" t="inlineStr">
         <is>
-          <t>via principal pavimentada</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y37" t="inlineStr">
@@ -5229,12 +5234,12 @@
       </c>
       <c r="Z37" t="inlineStr">
         <is>
-          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 12 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 10 m de esa vía.</t>
         </is>
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>Calle 27</t>
+          <t>Carrera 5</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
@@ -5243,10 +5248,10 @@
         </is>
       </c>
       <c r="AC37" t="n">
-        <v>4.088515899</v>
+        <v>4.412260842287796</v>
       </c>
       <c r="AD37" t="n">
-        <v>-76.22009</v>
+        <v>-76.15737540436542</v>
       </c>
     </row>
     <row r="38">
@@ -5281,74 +5286,74 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>JOSE MARIA CORDOBA</t>
+          <t>MANUEL DOLORES MONDRAGON</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA HERNANDO LLORENTE ARROYO</t>
+          <t>INSTITUCION EDUCATIVA MANUEL DOLORES MONDRAGON</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>276616000212</t>
+          <t>176100000254</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>RIOFRIO</t>
+          <t>BOLIVAR</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>CORREG SALONICA</t>
+          <t>KR 2 2 66</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
+          <t>Andalucia</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
           <t>Tulua</t>
         </is>
       </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>Tulua</t>
-        </is>
-      </c>
       <c r="P38" t="n">
-        <v>42.09</v>
+        <v>14.74</v>
       </c>
       <c r="Q38" t="n">
-        <v>50.65</v>
+        <v>50.86</v>
       </c>
       <c r="R38" t="n">
-        <v>100.2</v>
+        <v>114.3</v>
       </c>
       <c r="S38" t="n">
-        <v>57</v>
+        <v>93.2</v>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>Peligro de colapso</t>
+          <t>Uso restringido</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>en revisión de la mesa</t>
+          <t>aprobado por la mesa</t>
         </is>
       </c>
       <c r="V38" t="inlineStr">
         <is>
-          <t>Riesgo inminente de colapso</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X38" t="inlineStr">
@@ -5363,12 +5368,12 @@
       </c>
       <c r="Z38" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 26 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 43 m de esa vía.</t>
         </is>
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>SALONICA CRUCE CON VIA 23VL13-1 EN K44+300</t>
+          <t>BOLIVAR CRUCE CON VIA DE INVIAS 2302 EN TRAMO 23020 INICIO A 52m DE INICIO DE VIA 10023VL02B</t>
         </is>
       </c>
       <c r="AB38" t="inlineStr">
@@ -5377,10 +5382,10 @@
         </is>
       </c>
       <c r="AC38" t="n">
-        <v>4.1258314</v>
+        <v>4.340805</v>
       </c>
       <c r="AD38" t="n">
-        <v>-76.3722336</v>
+        <v>-76.17979800000001</v>
       </c>
     </row>
     <row r="39">
@@ -5410,27 +5415,27 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Tuluá</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>INTEGRADA DE TRUJILLO</t>
+          <t>SEDE PRINCIPAL LICEO MODERNO</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA INTEGRADA DE TRUJILLO</t>
+          <t>INSTITUCION EDUCATIVA MODERNA DE TULUA</t>
         </is>
       </c>
       <c r="J39" s="3" t="inlineStr">
         <is>
-          <t>176828000021</t>
+          <t>176834000106</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>TRUJILLO</t>
+          <t>Tuluá</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
@@ -5440,7 +5445,7 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>KR 18 15 40</t>
+          <t>IND CALLE 27 NO. 6AW 240</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -5454,40 +5459,30 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>46.98</v>
+        <v>7.41</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.67</v>
+        <v>42.09</v>
       </c>
       <c r="R39" t="n">
-        <v>91.90000000000001</v>
+        <v>100.2</v>
       </c>
       <c r="S39" t="n">
-        <v>48.5</v>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>No habitable</t>
-        </is>
-      </c>
-      <c r="U39" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
+        <v>57</v>
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X39" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>via principal pavimentada</t>
         </is>
       </c>
       <c r="Y39" t="inlineStr">
@@ -5497,12 +5492,12 @@
       </c>
       <c r="Z39" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 33 m de esa vía.</t>
+          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 12 m de esa vía.</t>
         </is>
       </c>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>Carrera 18</t>
+          <t>Calle 27</t>
         </is>
       </c>
       <c r="AB39" t="inlineStr">
@@ -5511,10 +5506,10 @@
         </is>
       </c>
       <c r="AC39" t="n">
-        <v>4.208406</v>
+        <v>4.088515899</v>
       </c>
       <c r="AD39" t="n">
-        <v>-76.31959500000001</v>
+        <v>-76.22009</v>
       </c>
     </row>
     <row r="40">
@@ -5549,32 +5544,32 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>SAGRADO CORAZON DE JESUS</t>
+          <t>JOSE MARIA CORDOBA</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA INTEGRADA DE TRUJILLO</t>
+          <t>INSTITUCION EDUCATIVA HERNANDO LLORENTE ARROYO</t>
         </is>
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>176828000064</t>
+          <t>276616000212</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>TRUJILLO</t>
+          <t>RIOFRIO</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>KR 18 15 27</t>
+          <t>CORREG SALONICA</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -5588,20 +5583,30 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>0.67</v>
+        <v>42.09</v>
       </c>
       <c r="Q40" t="n">
-        <v>44.3</v>
+        <v>50.65</v>
       </c>
       <c r="R40" t="n">
-        <v>91.90000000000001</v>
+        <v>100.2</v>
       </c>
       <c r="S40" t="n">
-        <v>48.5</v>
+        <v>57</v>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>Peligro de colapso</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>en revisión de la mesa</t>
+        </is>
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Riesgo inminente de colapso</t>
         </is>
       </c>
       <c r="W40" t="inlineStr">
@@ -5626,7 +5631,7 @@
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>Carrera 18</t>
+          <t>SALONICA CRUCE CON VIA 23VL13-1 EN K44+300</t>
         </is>
       </c>
       <c r="AB40" t="inlineStr">
@@ -5635,10 +5640,10 @@
         </is>
       </c>
       <c r="AC40" t="n">
-        <v>4.210077</v>
+        <v>4.1258314</v>
       </c>
       <c r="AD40" t="n">
-        <v>-76.319047</v>
+        <v>-76.3722336</v>
       </c>
     </row>
     <row r="41">
@@ -5673,17 +5678,17 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>SAN ISIDRO</t>
+          <t>INTEGRADA DE TRUJILLO</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA SAN ISIDRO</t>
+          <t>INSTITUCION EDUCATIVA INTEGRADA DE TRUJILLO</t>
         </is>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>276828000174</t>
+          <t>176828000021</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -5693,12 +5698,12 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>CORREGIMIENTO EL TABOR PUENTE BLANCO</t>
+          <t>KR 18 15 40</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -5712,20 +5717,20 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>77.20999999999999</v>
+        <v>46.98</v>
       </c>
       <c r="Q41" t="n">
-        <v>69.08</v>
+        <v>0.67</v>
       </c>
       <c r="R41" t="n">
-        <v>146.3</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="S41" t="n">
-        <v>74.2</v>
+        <v>48.5</v>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>Habitable</t>
+          <t>No habitable</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
@@ -5745,7 +5750,7 @@
       </c>
       <c r="X41" t="inlineStr">
         <is>
-          <t>via terciaria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr">
@@ -5755,12 +5760,12 @@
       </c>
       <c r="Z41" t="inlineStr">
         <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 33 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 33 m de esa vía.</t>
         </is>
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t>TRUJILLO - LA SONORA CRUCE VIA 23VL13-1 K64+160</t>
+          <t>Carrera 18</t>
         </is>
       </c>
       <c r="AB41" t="inlineStr">
@@ -5769,10 +5774,10 @@
         </is>
       </c>
       <c r="AC41" t="n">
-        <v>4.210564</v>
+        <v>4.208406</v>
       </c>
       <c r="AD41" t="n">
-        <v>-76.38158300000001</v>
+        <v>-76.31959500000001</v>
       </c>
     </row>
     <row r="42">
@@ -5787,42 +5792,42 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>lunes</t>
+          <t>sábado</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Tuluá</t>
+          <t>BID (43)</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>SEDE INSTITUTO CAMPESTRE SANTA CECILIA</t>
+          <t>SAGRADO CORAZON DE JESUS</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA MODERNA DE TULUA</t>
+          <t>INSTITUCION EDUCATIVA INTEGRADA DE TRUJILLO</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>176834000599</t>
+          <t>176828000064</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Tuluá</t>
+          <t>TRUJILLO</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
@@ -5832,7 +5837,7 @@
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>IND CALLE 27 NO 6AW 240</t>
+          <t>KR 18 15 27</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -5842,44 +5847,49 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>Yotoco</t>
+          <t>Tulua</t>
         </is>
       </c>
       <c r="P42" t="n">
-        <v>9.890000000000001</v>
+        <v>0.67</v>
       </c>
       <c r="Q42" t="n">
-        <v>32.44</v>
+        <v>44.3</v>
       </c>
       <c r="R42" t="n">
-        <v>82.5</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="S42" t="n">
-        <v>59.6</v>
+        <v>48.5</v>
       </c>
       <c r="V42" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X42" t="inlineStr">
         <is>
-          <t>camino destapado</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y42" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="Z42" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 50 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 26 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AA42" t="inlineStr">
+        <is>
+          <t>Carrera 18</t>
         </is>
       </c>
       <c r="AB42" t="inlineStr">
@@ -5888,10 +5898,10 @@
         </is>
       </c>
       <c r="AC42" t="n">
-        <v>4.090555556</v>
+        <v>4.210077</v>
       </c>
       <c r="AD42" t="n">
-        <v>-76.22221999999999</v>
+        <v>-76.319047</v>
       </c>
     </row>
     <row r="43">
@@ -5917,7 +5927,7 @@
         <v>13</v>
       </c>
       <c r="F43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -5926,22 +5936,22 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>ALFREDO GARRIDO TOVAR</t>
+          <t>SAN ISIDRO</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA ALFREDO GARRIDO TOVAR</t>
+          <t>INSTITUCION EDUCATIVA SAN ISIDRO</t>
         </is>
       </c>
       <c r="J43" s="3" t="inlineStr">
         <is>
-          <t>276616000654</t>
+          <t>276828000174</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>RIOFRIO</t>
+          <t>TRUJILLO</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -5951,7 +5961,7 @@
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>CORREG PORTUGAL DE PIEDRAS</t>
+          <t>CORREGIMIENTO EL TABOR PUENTE BLANCO</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -5961,24 +5971,24 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>Yotoco</t>
+          <t>Tulua</t>
         </is>
       </c>
       <c r="P43" t="n">
-        <v>32.44</v>
+        <v>77.20999999999999</v>
       </c>
       <c r="Q43" t="n">
-        <v>40.13</v>
+        <v>69.08</v>
       </c>
       <c r="R43" t="n">
-        <v>82.5</v>
+        <v>146.3</v>
       </c>
       <c r="S43" t="n">
-        <v>59.6</v>
+        <v>74.2</v>
       </c>
       <c r="T43" t="inlineStr">
         <is>
-          <t>No habitable</t>
+          <t>Habitable</t>
         </is>
       </c>
       <c r="U43" t="inlineStr">
@@ -5988,32 +5998,32 @@
       </c>
       <c r="V43" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X43" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="Z43" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 36 m de esa vía.</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 33 m de esa vía.</t>
         </is>
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>PORTUGAL DE PIEDRAS - CRUCE VIA 23VL13</t>
+          <t>TRUJILLO - LA SONORA CRUCE VIA 23VL13-1 K64+160</t>
         </is>
       </c>
       <c r="AB43" t="inlineStr">
@@ -6022,10 +6032,10 @@
         </is>
       </c>
       <c r="AC43" t="n">
-        <v>4.0553</v>
+        <v>4.210564</v>
       </c>
       <c r="AD43" t="n">
-        <v>-76.35465000000001</v>
+        <v>-76.38158300000001</v>
       </c>
     </row>
     <row r="44">
@@ -6055,27 +6065,27 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Tuluá</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>ALFONSO ZAWADZKY</t>
+          <t>SEDE INSTITUTO CAMPESTRE SANTA CECILIA</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA ALFONSO ZAWADZKY</t>
+          <t>INSTITUCION EDUCATIVA MODERNA DE TULUA</t>
         </is>
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>176890000305</t>
+          <t>176834000599</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>YOTOCO</t>
+          <t>Tuluá</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
@@ -6085,12 +6095,12 @@
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>KR 5 5 79</t>
+          <t>IND CALLE 27 NO 6AW 240</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Yotoco</t>
+          <t>Tulua</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -6099,40 +6109,30 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>0.76</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="Q44" t="n">
-        <v>23.14</v>
+        <v>32.44</v>
       </c>
       <c r="R44" t="n">
-        <v>25.1</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="S44" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="T44" t="inlineStr">
-        <is>
-          <t>No habitable</t>
-        </is>
-      </c>
-      <c r="U44" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
+        <v>62</v>
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>Riesgo inminente de colapso</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="X44" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>camino destapado</t>
         </is>
       </c>
       <c r="Y44" t="inlineStr">
@@ -6142,12 +6142,7 @@
       </c>
       <c r="Z44" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 15 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA44" t="inlineStr">
-        <is>
-          <t>Calle 6</t>
+          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 50 m de esa vía.</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -6156,10 +6151,10 @@
         </is>
       </c>
       <c r="AC44" t="n">
-        <v>3.86056963997</v>
+        <v>4.090555556</v>
       </c>
       <c r="AD44" t="n">
-        <v>-76.38430955440001</v>
+        <v>-76.22221999999999</v>
       </c>
     </row>
     <row r="45">
@@ -6189,89 +6184,99 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
+          <t>BID (43)</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>ALFREDO GARRIDO TOVAR</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>INSTITUCION EDUCATIVA ALFREDO GARRIDO TOVAR</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>276616000654</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>RIOFRIO</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Rural</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>CORREG PORTUGAL DE PIEDRAS</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>Tulua</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
           <t>Buga</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>EL PLACER - SEDE PRINCIPAL</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>INSTITUCION EDUCATIVA EL PLACER</t>
-        </is>
-      </c>
-      <c r="J45" s="3" t="inlineStr">
-        <is>
-          <t>276111000102</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>Buga</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>Rural</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr">
-        <is>
-          <t>CORREG EL PLACER</t>
-        </is>
-      </c>
-      <c r="N45" t="inlineStr">
-        <is>
-          <t>Yotoco</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
-        <is>
-          <t>Buga</t>
-        </is>
-      </c>
       <c r="P45" t="n">
-        <v>23.14</v>
+        <v>32.44</v>
       </c>
       <c r="Q45" t="n">
-        <v>1.2</v>
+        <v>47.02</v>
       </c>
       <c r="R45" t="n">
-        <v>25.1</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="S45" t="n">
-        <v>13.6</v>
+        <v>62</v>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>No habitable</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>aprobado por la mesa</t>
+        </is>
       </c>
       <c r="V45" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X45" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>camino rural sin categoria</t>
         </is>
       </c>
       <c r="Y45" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="Z45" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 30 m de esa vía.</t>
+          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 36 m de esa vía.</t>
         </is>
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>Calle 6</t>
+          <t>PORTUGAL DE PIEDRAS - CRUCE VIA 23VL13</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -6280,10 +6285,10 @@
         </is>
       </c>
       <c r="AC45" t="n">
-        <v>3.898611</v>
+        <v>4.0553</v>
       </c>
       <c r="AD45" t="n">
-        <v>-76.30056</v>
+        <v>-76.35465000000001</v>
       </c>
     </row>
     <row r="46">
@@ -6318,17 +6323,17 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>ACADEMICO - SEDE PRINCIPAL</t>
+          <t>TULIO ENRIQUE TASCON CHAMBIMBAL - SEDE PRINCIPAL</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA ACADEMICO</t>
+          <t>INSTITUCION EDUCATIVA TULIO ENRIQUE TASCON CHAMBIMBAL</t>
         </is>
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>176111001104</t>
+          <t>276111000781</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -6338,12 +6343,12 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>KR 9 A 2 55 SUR</t>
+          <t>CHAMBIMBAL</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -6357,16 +6362,16 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>3.44</v>
+        <v>24.58</v>
       </c>
       <c r="Q46" t="n">
-        <v>13.01</v>
+        <v>24.3</v>
       </c>
       <c r="R46" t="n">
-        <v>84.3</v>
+        <v>116.8</v>
       </c>
       <c r="S46" t="n">
-        <v>69.09999999999999</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="V46" t="inlineStr">
         <is>
@@ -6380,22 +6385,17 @@
       </c>
       <c r="X46" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>camino rural sin categoria</t>
         </is>
       </c>
       <c r="Y46" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="Z46" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 25 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA46" t="inlineStr">
-        <is>
-          <t>Carrera 9</t>
+          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 187 m de esa vía.</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -6404,10 +6404,10 @@
         </is>
       </c>
       <c r="AC46" t="n">
-        <v>3.892781656</v>
+        <v>3.956111</v>
       </c>
       <c r="AD46" t="n">
-        <v>-76.29845</v>
+        <v>-76.30028</v>
       </c>
     </row>
     <row r="47">
@@ -6481,16 +6481,16 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>13.01</v>
+        <v>24.3</v>
       </c>
       <c r="Q47" t="n">
         <v>67.88</v>
       </c>
       <c r="R47" t="n">
-        <v>84.3</v>
+        <v>116.8</v>
       </c>
       <c r="S47" t="n">
-        <v>69.09999999999999</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="V47" t="inlineStr">
         <is>
@@ -12183,10 +12183,10 @@
         <v>28</v>
       </c>
       <c r="D11" t="n">
-        <v>20.1</v>
+        <v>19</v>
       </c>
       <c r="E11" t="n">
-        <v>822</v>
+        <v>747</v>
       </c>
       <c r="F11" t="n">
         <v>14</v>

</xml_diff>

<commit_message>
Santo Tomas de Aquino (Palmira) en su predio; Valle 101,4 h
La sede queda en el predio «ESCUELA SANTO TOMAS DE AQUINO» del catastro, a 283 m
del punto del SIMAT, confirmado con fotos de la escuela en la vereda El Meson. El
plan del Valle pasa de 101,23 h a 101,38 h con el mismo reparto.
</commit_message>
<xml_diff>
--- a/public/datos/plan_cuadrillas_todas_4_cuadrillas.xlsx
+++ b/public/datos/plan_cuadrillas_todas_4_cuadrillas.xlsx
@@ -9602,32 +9602,32 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>JOSE EUSEBIO CARO</t>
+          <t>SAGRADO CORAZON DE JESUS</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA INMACULADA CONCEPCION</t>
+          <t>INSTITUCION EDUCATIVA ABSALON TORRES CAMACHO</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>276130000288</t>
+          <t>176275000125</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>CANDELARIA</t>
+          <t>FLORIDA</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>CR 12 NO 10-81</t>
+          <t>CR 21 NO 9-89</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -9641,26 +9641,16 @@
         </is>
       </c>
       <c r="P72" t="n">
-        <v>11.66</v>
+        <v>27.65</v>
       </c>
       <c r="Q72" t="n">
-        <v>8.539999999999999</v>
+        <v>28.95</v>
       </c>
       <c r="R72" t="n">
-        <v>20.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="S72" t="n">
-        <v>13.6</v>
-      </c>
-      <c r="T72" t="inlineStr">
-        <is>
-          <t>No habitable</t>
-        </is>
-      </c>
-      <c r="U72" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
+        <v>44</v>
       </c>
       <c r="V72" t="inlineStr">
         <is>
@@ -9684,12 +9674,12 @@
       </c>
       <c r="Z72" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 1 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 23 m de esa vía.</t>
         </is>
       </c>
       <c r="AA72" t="inlineStr">
         <is>
-          <t>CALLEJON FLORO MERCADO CRUCE VIA 13025VL04-2E</t>
+          <t>Calle 10</t>
         </is>
       </c>
       <c r="AB72" t="inlineStr">
@@ -9698,10 +9688,10 @@
         </is>
       </c>
       <c r="AC72" t="n">
-        <v>3.39537597879</v>
+        <v>3.32644406118</v>
       </c>
       <c r="AD72" t="n">
-        <v>-76.3859481842</v>
+        <v>-76.23742270629999</v>
       </c>
     </row>
     <row r="73">
@@ -9720,14 +9710,14 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>jueves</t>
+          <t>miércoles</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>
@@ -9736,32 +9726,32 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>SAGRADO CORAZON DE JESUS</t>
+          <t>JOSE EUSEBIO CARO</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA ABSALON TORRES CAMACHO</t>
+          <t>INSTITUCION EDUCATIVA INMACULADA CONCEPCION</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>176275000125</t>
+          <t>276130000288</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>FLORIDA</t>
+          <t>CANDELARIA</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>CR 21 NO 9-89</t>
+          <t>CR 12 NO 10-81</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -9771,20 +9761,30 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="P73" t="n">
-        <v>27.65</v>
+        <v>28.95</v>
       </c>
       <c r="Q73" t="n">
-        <v>50.58</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="R73" t="n">
-        <v>119.1</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="S73" t="n">
-        <v>65.8</v>
+        <v>44</v>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>No habitable</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>aprobado por la mesa</t>
+        </is>
       </c>
       <c r="V73" t="inlineStr">
         <is>
@@ -9808,12 +9808,12 @@
       </c>
       <c r="Z73" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 23 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 1 m de esa vía.</t>
         </is>
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>Calle 10</t>
+          <t>CALLEJON FLORO MERCADO CRUCE VIA 13025VL04-2E</t>
         </is>
       </c>
       <c r="AB73" t="inlineStr">
@@ -9822,10 +9822,10 @@
         </is>
       </c>
       <c r="AC73" t="n">
-        <v>3.32644406118</v>
+        <v>3.39537597879</v>
       </c>
       <c r="AD73" t="n">
-        <v>-76.23742270629999</v>
+        <v>-76.3859481842</v>
       </c>
     </row>
     <row r="74">
@@ -9851,7 +9851,7 @@
         <v>4</v>
       </c>
       <c r="F74" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G74" t="inlineStr">
         <is>
@@ -9899,16 +9899,16 @@
         </is>
       </c>
       <c r="P74" t="n">
-        <v>50.58</v>
+        <v>60.37</v>
       </c>
       <c r="Q74" t="n">
-        <v>40.86</v>
+        <v>40.02</v>
       </c>
       <c r="R74" t="n">
-        <v>119.1</v>
+        <v>117.8</v>
       </c>
       <c r="S74" t="n">
-        <v>65.8</v>
+        <v>61.6</v>
       </c>
       <c r="V74" t="inlineStr">
         <is>
@@ -9932,19 +9932,19 @@
       </c>
       <c r="Z74" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 129 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 35 m de esa vía.</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AC74" t="n">
-        <v>3.499130225</v>
+        <v>3.496808</v>
       </c>
       <c r="AD74" t="n">
-        <v>-76.18842022</v>
+        <v>-76.189471</v>
       </c>
     </row>
     <row r="75">
@@ -9963,14 +9963,14 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F75" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G75" t="inlineStr">
         <is>
@@ -9979,17 +9979,17 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>NIÑA MARIA</t>
+          <t>ROSARIO DE FATIMA</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DEL PALMAR</t>
+          <t>INSTITUCION EDUCATIVA TABLONES</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>176520002261</t>
+          <t>276520000742</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -9999,76 +9999,76 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>KR 26 37 01</t>
+          <t>CORREG LA BOLSA</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
         <is>
+          <t>Candelaria</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
           <t>Palmira</t>
         </is>
       </c>
-      <c r="O75" t="inlineStr">
-        <is>
-          <t>Palmira</t>
-        </is>
-      </c>
       <c r="P75" t="n">
-        <v>1.99</v>
+        <v>40.02</v>
       </c>
       <c r="Q75" t="n">
-        <v>1.75</v>
+        <v>17.42</v>
       </c>
       <c r="R75" t="n">
-        <v>6.4</v>
+        <v>117.8</v>
       </c>
       <c r="S75" t="n">
-        <v>1.9</v>
+        <v>61.6</v>
       </c>
       <c r="V75" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>camino destapado</t>
         </is>
       </c>
       <c r="Y75" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="Z75" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 21 m de esa vía.</t>
+          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 18 m de esa vía.</t>
         </is>
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>Carrera 26</t>
+          <t>La Bolsa</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AC75" t="n">
-        <v>3.53399314013</v>
+        <v>3.555961</v>
       </c>
       <c r="AD75" t="n">
-        <v>-76.2962377697</v>
+        <v>-76.23436599999999</v>
       </c>
     </row>
     <row r="76">
@@ -10094,7 +10094,7 @@
         <v>5</v>
       </c>
       <c r="F76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G76" t="inlineStr">
         <is>
@@ -10103,7 +10103,7 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>LICEO FEMENINO</t>
+          <t>NIÑA MARIA</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -10113,7 +10113,7 @@
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>176520000489</t>
+          <t>176520002261</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -10128,7 +10128,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>CR 28 NO 37 81</t>
+          <t>KR 26 37 01</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -10142,16 +10142,16 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>1.75</v>
+        <v>1.99</v>
       </c>
       <c r="Q76" t="n">
-        <v>2.66</v>
+        <v>2.01</v>
       </c>
       <c r="R76" t="n">
-        <v>6.4</v>
+        <v>4</v>
       </c>
       <c r="S76" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="V76" t="inlineStr">
         <is>
@@ -10165,7 +10165,7 @@
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>via principal pavimentada</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="Y76" t="inlineStr">
@@ -10175,12 +10175,12 @@
       </c>
       <c r="Z76" t="inlineStr">
         <is>
-          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 43 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 21 m de esa vía.</t>
         </is>
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t>Carrera 28</t>
+          <t>Carrera 26</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -10189,10 +10189,10 @@
         </is>
       </c>
       <c r="AC76" t="n">
-        <v>3.53438389943</v>
+        <v>3.53399314013</v>
       </c>
       <c r="AD76" t="n">
-        <v>-76.2982293309</v>
+        <v>-76.2962377697</v>
       </c>
     </row>
     <row r="77">
@@ -10760,13 +10760,13 @@
         <v>10.39</v>
       </c>
       <c r="Q81" t="n">
-        <v>47.5</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="R81" t="n">
-        <v>100.6</v>
+        <v>21.8</v>
       </c>
       <c r="S81" t="n">
-        <v>55.7</v>
+        <v>7.6</v>
       </c>
       <c r="V81" t="inlineStr">
         <is>
@@ -10842,17 +10842,17 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>MARCO FIDEL SUAREZ</t>
+          <t>LICEO FEMENINO</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA TABLONES</t>
+          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DEL PALMAR</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>276520001684</t>
+          <t>176520000489</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -10862,12 +10862,12 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>VDA LA ESPERANZA</t>
+          <t>CR 28 NO 37 81</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -10881,20 +10881,30 @@
         </is>
       </c>
       <c r="P82" t="n">
-        <v>47.5</v>
+        <v>8.789999999999999</v>
       </c>
       <c r="Q82" t="n">
-        <v>42.74</v>
+        <v>2.66</v>
       </c>
       <c r="R82" t="n">
-        <v>100.6</v>
+        <v>21.8</v>
       </c>
       <c r="S82" t="n">
-        <v>55.7</v>
+        <v>7.6</v>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>Afectación parcial</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
       </c>
       <c r="X82" t="inlineStr">
         <is>
-          <t>via terciaria</t>
+          <t>via principal pavimentada</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr">
@@ -10904,19 +10914,24 @@
       </c>
       <c r="Z82" t="inlineStr">
         <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 9 m de esa vía.</t>
+          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 43 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AA82" t="inlineStr">
+        <is>
+          <t>Carrera 28</t>
         </is>
       </c>
       <c r="AB82" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="AC82" t="n">
-        <v>3.610511</v>
+        <v>3.53438389943</v>
       </c>
       <c r="AD82" t="n">
-        <v>-76.155193</v>
+        <v>-76.2982293309</v>
       </c>
     </row>
     <row r="83">
@@ -10993,13 +11008,13 @@
         <v>33.72</v>
       </c>
       <c r="Q83" t="n">
-        <v>2.14</v>
+        <v>22.95</v>
       </c>
       <c r="R83" t="n">
-        <v>53.3</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="S83" t="n">
-        <v>28.7</v>
+        <v>56.1</v>
       </c>
       <c r="V83" t="inlineStr">
         <is>
@@ -11075,7 +11090,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>ROSARIO DE FATIMA</t>
+          <t>MARCO FIDEL SUAREZ</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -11085,7 +11100,7 @@
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>276520000742</t>
+          <t>276520001684</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -11100,7 +11115,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>CORREG LA BOLSA</t>
+          <t>VDA LA ESPERANZA</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -11114,45 +11129,30 @@
         </is>
       </c>
       <c r="P84" t="n">
-        <v>2.14</v>
+        <v>22.95</v>
       </c>
       <c r="Q84" t="n">
-        <v>17.42</v>
+        <v>42.74</v>
       </c>
       <c r="R84" t="n">
-        <v>53.3</v>
+        <v>99.40000000000001</v>
       </c>
       <c r="S84" t="n">
-        <v>28.7</v>
-      </c>
-      <c r="V84" t="inlineStr">
-        <is>
-          <t>Colapso parcial</t>
-        </is>
-      </c>
-      <c r="W84" t="inlineStr">
-        <is>
-          <t>Critico</t>
-        </is>
+        <v>56.1</v>
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>camino destapado</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="Y84" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="Z84" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 18 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AA84" t="inlineStr">
-        <is>
-          <t>La Bolsa</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 9 m de esa vía.</t>
         </is>
       </c>
       <c r="AB84" t="inlineStr">
@@ -11161,10 +11161,10 @@
         </is>
       </c>
       <c r="AC84" t="n">
-        <v>3.555961</v>
+        <v>3.610511</v>
       </c>
       <c r="AD84" t="n">
-        <v>-76.23436599999999</v>
+        <v>-76.155193</v>
       </c>
     </row>
     <row r="85">
@@ -12223,10 +12223,10 @@
         <v>24</v>
       </c>
       <c r="D13" t="n">
-        <v>18.8</v>
+        <v>18.9</v>
       </c>
       <c r="E13" t="n">
-        <v>567</v>
+        <v>572</v>
       </c>
       <c r="F13" t="n">
         <v>13</v>

</xml_diff>

<commit_message>
Palmira con la respuesta de su Secretaria y Risaralda solo desde Pereira
- Valle: salen Maria Dominguez y Marco Fidel Suarez, entran Rosa Virginia y
  Rosa Zarate de Pena, y cinco sedes de Palmira pasan a la coordenada que
  mando su Secretaria. El plan baja de 101,4 h a 97,5 h de carretera, con
  las mismas 90 sedes y 58 dias.
- Risaralda: fuera el traslado de las cuadrillas desde Armenia y el plan con
  los puntos corroborados del 1-oct.
</commit_message>
<xml_diff>
--- a/public/datos/plan_cuadrillas_todas_4_cuadrillas.xlsx
+++ b/public/datos/plan_cuadrillas_todas_4_cuadrillas.xlsx
@@ -9631,7 +9631,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="P68" t="n">
@@ -9641,10 +9641,10 @@
         <v>7.07</v>
       </c>
       <c r="R68" t="n">
-        <v>83.3</v>
+        <v>75.8</v>
       </c>
       <c r="S68" t="n">
-        <v>61.9</v>
+        <v>49.8</v>
       </c>
       <c r="X68" t="inlineStr">
         <is>
@@ -9755,20 +9755,20 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="P69" t="n">
         <v>7.07</v>
       </c>
       <c r="Q69" t="n">
-        <v>37.84</v>
+        <v>30.35</v>
       </c>
       <c r="R69" t="n">
-        <v>83.3</v>
+        <v>75.8</v>
       </c>
       <c r="S69" t="n">
-        <v>61.9</v>
+        <v>49.8</v>
       </c>
       <c r="X69" t="inlineStr">
         <is>
@@ -9839,27 +9839,27 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>ALFONSO LOPEZ PUMAREJO</t>
+          <t>NIÑA MARIA</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DE LA CANDELARIA</t>
+          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DEL PALMAR</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>176130000330</t>
+          <t>176520002261</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>CANDELARIA</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
@@ -9869,45 +9869,30 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>CL 7 9 11</t>
+          <t>KR 26 37 01</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="P70" t="n">
-        <v>0.23</v>
+        <v>1.99</v>
       </c>
       <c r="Q70" t="n">
-        <v>0.25</v>
+        <v>1.75</v>
       </c>
       <c r="R70" t="n">
-        <v>2.2</v>
+        <v>6.4</v>
       </c>
       <c r="S70" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="T70" t="inlineStr">
-        <is>
-          <t>PATOLOGIA ESTRUCTURAL</t>
-        </is>
-      </c>
-      <c r="U70" t="inlineStr">
-        <is>
-          <t>No habitable</t>
-        </is>
-      </c>
-      <c r="V70" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
+        <v>1.9</v>
       </c>
       <c r="X70" t="inlineStr">
         <is>
@@ -9919,14 +9904,9 @@
           <t>Moderado</t>
         </is>
       </c>
-      <c r="Z70" t="inlineStr">
-        <is>
-          <t>Afectación parcial</t>
-        </is>
-      </c>
       <c r="AC70" t="inlineStr">
         <is>
-          <t>via terciaria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="AD70" t="inlineStr">
@@ -9936,24 +9916,24 @@
       </c>
       <c r="AE70" t="inlineStr">
         <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 2 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 21 m de esa vía.</t>
         </is>
       </c>
       <c r="AF70" t="inlineStr">
         <is>
-          <t>Calle 7</t>
+          <t>Carrera 26</t>
         </is>
       </c>
       <c r="AG70" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="AH70" t="n">
-        <v>3.407489</v>
+        <v>3.53399314013</v>
       </c>
       <c r="AI70" t="n">
-        <v>-76.34917799999999</v>
+        <v>-76.2962377697</v>
       </c>
     </row>
     <row r="71">
@@ -9983,27 +9963,27 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>SAGRADA FAMILIA</t>
+          <t>LICEO FEMENINO</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DE LA CANDELARIA</t>
+          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DEL PALMAR</t>
         </is>
       </c>
       <c r="J71" s="3" t="inlineStr">
         <is>
-          <t>176130000356</t>
+          <t>176520000489</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>CANDELARIA</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
@@ -10013,45 +9993,30 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>CL 7 8 42</t>
+          <t>CR 28 NO 37 81</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="P71" t="n">
-        <v>0.25</v>
+        <v>1.75</v>
       </c>
       <c r="Q71" t="n">
-        <v>1.68</v>
+        <v>2.66</v>
       </c>
       <c r="R71" t="n">
-        <v>2.2</v>
+        <v>6.4</v>
       </c>
       <c r="S71" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="T71" t="inlineStr">
-        <is>
-          <t>PATOLOGIA ESTRUCTURAL</t>
-        </is>
-      </c>
-      <c r="U71" t="inlineStr">
-        <is>
-          <t>No habitable</t>
-        </is>
-      </c>
-      <c r="V71" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
+        <v>1.9</v>
       </c>
       <c r="X71" t="inlineStr">
         <is>
@@ -10063,14 +10028,9 @@
           <t>Moderado</t>
         </is>
       </c>
-      <c r="Z71" t="inlineStr">
-        <is>
-          <t>Afectación parcial</t>
-        </is>
-      </c>
       <c r="AC71" t="inlineStr">
         <is>
-          <t>via terciaria</t>
+          <t>via principal pavimentada</t>
         </is>
       </c>
       <c r="AD71" t="inlineStr">
@@ -10080,24 +10040,24 @@
       </c>
       <c r="AE71" t="inlineStr">
         <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 33 m de esa vía.</t>
+          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 43 m de esa vía.</t>
         </is>
       </c>
       <c r="AF71" t="inlineStr">
         <is>
-          <t>Calle 7</t>
+          <t>Carrera 28</t>
         </is>
       </c>
       <c r="AG71" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="AH71" t="n">
-        <v>3.40761667</v>
+        <v>3.53438389943</v>
       </c>
       <c r="AI71" t="n">
-        <v>-76.34858894</v>
+        <v>-76.2982293309</v>
       </c>
     </row>
     <row r="72">
@@ -10127,27 +10087,27 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>SAGRADO CORAZON DE JESUS</t>
+          <t>ROSA VIRGINIA</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA ABSALON TORRES CAMACHO</t>
+          <t>INSTITUCION EDUCATIVA SAN VICENTE</t>
         </is>
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>176275000125</t>
+          <t>176520002295</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>FLORIDA</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
@@ -10157,35 +10117,30 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>CR 21 NO 9-89</t>
+          <t>CR 32 NO 46 00</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="P72" t="n">
-        <v>27.65</v>
+        <v>5.2</v>
       </c>
       <c r="Q72" t="n">
-        <v>28.95</v>
+        <v>7.79</v>
       </c>
       <c r="R72" t="n">
-        <v>65.09999999999999</v>
+        <v>18.9</v>
       </c>
       <c r="S72" t="n">
-        <v>44</v>
-      </c>
-      <c r="T72" t="inlineStr">
-        <is>
-          <t>PATOLOGIA ESTRUCTURAL</t>
-        </is>
+        <v>6.3</v>
       </c>
       <c r="X72" t="inlineStr">
         <is>
@@ -10209,12 +10164,12 @@
       </c>
       <c r="AE72" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 23 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 5 m de esa vía.</t>
         </is>
       </c>
       <c r="AF72" t="inlineStr">
         <is>
-          <t>Calle 10</t>
+          <t>Calle 46</t>
         </is>
       </c>
       <c r="AG72" t="inlineStr">
@@ -10223,10 +10178,10 @@
         </is>
       </c>
       <c r="AH72" t="n">
-        <v>3.32644406118</v>
+        <v>3.541522</v>
       </c>
       <c r="AI72" t="n">
-        <v>-76.23742270629999</v>
+        <v>-76.300059</v>
       </c>
     </row>
     <row r="73">
@@ -10256,75 +10211,60 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>BID (43)</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>JOSE EUSEBIO CARO</t>
+          <t>ENELIA RIVERA</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA INMACULADA CONCEPCION</t>
+          <t>INSTITUCION EDUCATIVA SANTA BARBARA</t>
         </is>
       </c>
       <c r="J73" s="3" t="inlineStr">
         <is>
-          <t>276130000288</t>
+          <t>176520001957</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>CANDELARIA</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>CR 12 NO 10-81</t>
+          <t>CLL 30 CR 40</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="P73" t="n">
-        <v>28.95</v>
+        <v>7.79</v>
       </c>
       <c r="Q73" t="n">
-        <v>8.539999999999999</v>
+        <v>5.87</v>
       </c>
       <c r="R73" t="n">
-        <v>65.09999999999999</v>
+        <v>18.9</v>
       </c>
       <c r="S73" t="n">
-        <v>44</v>
-      </c>
-      <c r="T73" t="inlineStr">
-        <is>
-          <t>PATOLOGIA ESTRUCTURAL</t>
-        </is>
-      </c>
-      <c r="U73" t="inlineStr">
-        <is>
-          <t>No habitable</t>
-        </is>
-      </c>
-      <c r="V73" t="inlineStr">
-        <is>
-          <t>aprobado por la mesa</t>
-        </is>
+        <v>6.3</v>
       </c>
       <c r="X73" t="inlineStr">
         <is>
@@ -10336,11 +10276,6 @@
           <t>Bajo</t>
         </is>
       </c>
-      <c r="Z73" t="inlineStr">
-        <is>
-          <t>Afectación menor</t>
-        </is>
-      </c>
       <c r="AC73" t="inlineStr">
         <is>
           <t>calle de casco urbano</t>
@@ -10353,24 +10288,24 @@
       </c>
       <c r="AE73" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 1 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 48 m de esa vía.</t>
         </is>
       </c>
       <c r="AF73" t="inlineStr">
         <is>
-          <t>CALLEJON FLORO MERCADO CRUCE VIA 13025VL04-2E</t>
+          <t>Carrera 41</t>
         </is>
       </c>
       <c r="AG73" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="AH73" t="n">
-        <v>3.39537597879</v>
+        <v>3.528369858</v>
       </c>
       <c r="AI73" t="n">
-        <v>-76.3859481842</v>
+        <v>-76.30969955</v>
       </c>
     </row>
     <row r="74">
@@ -10405,17 +10340,17 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>SANTO TOMAS DE AQUINO</t>
+          <t>CENTRO ALFONSO LOPEZ</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA FRANCISCO MIRANDA</t>
+          <t>INSTITUCION EDUCATIVA DOMINGO IRURITA</t>
         </is>
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>276520000548</t>
+          <t>176520003623</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -10425,17 +10360,17 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>VDA MESON</t>
+          <t>KR 25 21 52</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="O74" t="inlineStr">
@@ -10444,25 +10379,25 @@
         </is>
       </c>
       <c r="P74" t="n">
-        <v>60.37</v>
+        <v>4.81</v>
       </c>
       <c r="Q74" t="n">
-        <v>40.02</v>
+        <v>3.85</v>
       </c>
       <c r="R74" t="n">
-        <v>117.8</v>
+        <v>14.4</v>
       </c>
       <c r="S74" t="n">
-        <v>61.6</v>
+        <v>4.5</v>
       </c>
       <c r="X74" t="inlineStr">
         <is>
-          <t>No reportó al MEN</t>
-        </is>
-      </c>
-      <c r="AB74" t="inlineStr">
-        <is>
-          <t>Sin concepto técnico ni reporte del rector</t>
+          <t>Afectación parcial</t>
+        </is>
+      </c>
+      <c r="Y74" t="inlineStr">
+        <is>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="AC74" t="inlineStr">
@@ -10477,7 +10412,12 @@
       </c>
       <c r="AE74" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 35 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 36 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AF74" t="inlineStr">
+        <is>
+          <t>Calle 21</t>
         </is>
       </c>
       <c r="AG74" t="inlineStr">
@@ -10486,10 +10426,10 @@
         </is>
       </c>
       <c r="AH74" t="n">
-        <v>3.496808</v>
+        <v>3.519487</v>
       </c>
       <c r="AI74" t="n">
-        <v>-76.189471</v>
+        <v>-76.29709</v>
       </c>
     </row>
     <row r="75">
@@ -10524,17 +10464,17 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>ROSARIO DE FATIMA</t>
+          <t>DOMINGO IRURITA</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA TABLONES</t>
+          <t>INSTITUCION EDUCATIVA DOMINGO IRURITA</t>
         </is>
       </c>
       <c r="J75" s="3" t="inlineStr">
         <is>
-          <t>276520000742</t>
+          <t>176520002163</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -10544,17 +10484,17 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>CORREG LA BOLSA</t>
+          <t>CL 23 33 A 37</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>Candelaria</t>
+          <t>Palmira</t>
         </is>
       </c>
       <c r="O75" t="inlineStr">
@@ -10563,57 +10503,57 @@
         </is>
       </c>
       <c r="P75" t="n">
-        <v>40.02</v>
+        <v>3.85</v>
       </c>
       <c r="Q75" t="n">
-        <v>17.42</v>
+        <v>5.78</v>
       </c>
       <c r="R75" t="n">
-        <v>117.8</v>
+        <v>14.4</v>
       </c>
       <c r="S75" t="n">
-        <v>61.6</v>
+        <v>4.5</v>
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>Colapso parcial</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="Y75" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="AC75" t="inlineStr">
         <is>
-          <t>camino destapado</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="AD75" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="AE75" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 18 m de esa vía.</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 35 m de esa vía.</t>
         </is>
       </c>
       <c r="AF75" t="inlineStr">
         <is>
-          <t>La Bolsa</t>
+          <t>Carrera 33A</t>
         </is>
       </c>
       <c r="AG75" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>sí</t>
         </is>
       </c>
       <c r="AH75" t="n">
-        <v>3.555961</v>
+        <v>3.521358245</v>
       </c>
       <c r="AI75" t="n">
-        <v>-76.23436599999999</v>
+        <v>-76.30535072000001</v>
       </c>
     </row>
     <row r="76">
@@ -10648,17 +10588,17 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>NIÑA MARIA</t>
+          <t>JOSE MANUEL GROOT</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DEL PALMAR</t>
+          <t>INSTITUCION EDUCATIVA HAROLD EDER</t>
         </is>
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>176520002261</t>
+          <t>276520002192</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -10673,7 +10613,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>KR 26 37 01</t>
+          <t>CL 65 31 C 95</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -10687,25 +10627,25 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>1.99</v>
+        <v>10.39</v>
       </c>
       <c r="Q76" t="n">
-        <v>2.01</v>
+        <v>3.11</v>
       </c>
       <c r="R76" t="n">
-        <v>4</v>
+        <v>25.3</v>
       </c>
       <c r="S76" t="n">
-        <v>1.2</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="X76" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Riesgo inminente de colapso</t>
         </is>
       </c>
       <c r="Y76" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="AC76" t="inlineStr">
@@ -10720,24 +10660,24 @@
       </c>
       <c r="AE76" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 21 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 2 m de esa vía.</t>
         </is>
       </c>
       <c r="AF76" t="inlineStr">
         <is>
-          <t>Carrera 26</t>
+          <t>Carrera 32</t>
         </is>
       </c>
       <c r="AG76" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AH76" t="n">
-        <v>3.53399314013</v>
+        <v>3.556083</v>
       </c>
       <c r="AI76" t="n">
-        <v>-76.2962377697</v>
+        <v>-76.30073299999999</v>
       </c>
     </row>
     <row r="77">
@@ -10756,14 +10696,14 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>sábado</t>
+          <t>viernes</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G77" t="inlineStr">
         <is>
@@ -10772,17 +10712,17 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>CENTRO ALFONSO LOPEZ</t>
+          <t>ROSA ZARATE DE PEÑA</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA DOMINGO IRURITA</t>
+          <t>INSTITUCION EDUCATIVA ANTONIO LIZARAZO</t>
         </is>
       </c>
       <c r="J77" s="3" t="inlineStr">
         <is>
-          <t>176520003623</t>
+          <t>276520001579</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -10797,7 +10737,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>KR 25 21 52</t>
+          <t>CL 63 30 06</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -10811,30 +10751,30 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>4.81</v>
+        <v>3.11</v>
       </c>
       <c r="Q77" t="n">
-        <v>7.64</v>
+        <v>11.82</v>
       </c>
       <c r="R77" t="n">
-        <v>19.5</v>
+        <v>25.3</v>
       </c>
       <c r="S77" t="n">
-        <v>5.8</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="X77" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
-        </is>
-      </c>
-      <c r="Y77" t="inlineStr">
-        <is>
-          <t>Moderado</t>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB77" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
         </is>
       </c>
       <c r="AC77" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="AD77" t="inlineStr">
@@ -10844,12 +10784,12 @@
       </c>
       <c r="AE77" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 36 m de esa vía.</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 6 m de esa vía.</t>
         </is>
       </c>
       <c r="AF77" t="inlineStr">
         <is>
-          <t>Calle 21</t>
+          <t>Calle 64</t>
         </is>
       </c>
       <c r="AG77" t="inlineStr">
@@ -10858,10 +10798,10 @@
         </is>
       </c>
       <c r="AH77" t="n">
-        <v>3.519487</v>
+        <v>3.553627286451045</v>
       </c>
       <c r="AI77" t="n">
-        <v>-76.29709</v>
+        <v>-76.30865764715436</v>
       </c>
     </row>
     <row r="78">
@@ -10887,7 +10827,7 @@
         <v>6</v>
       </c>
       <c r="F78" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -10896,17 +10836,17 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>ALFONSO LOPEZ PUMAREJO</t>
+          <t>CRISTOBAL COLON</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA ALFONSO LOPEZ PUMAREJO</t>
+          <t>INSTITUCION EDUCATIVA TABLONES</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>176520002091</t>
+          <t>276520001552</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -10916,12 +10856,12 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>KR 16 32 02</t>
+          <t>VDA LA CASCADA</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -10935,30 +10875,30 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>7.64</v>
+        <v>33.72</v>
       </c>
       <c r="Q78" t="n">
-        <v>7.03</v>
+        <v>2.14</v>
       </c>
       <c r="R78" t="n">
-        <v>19.5</v>
+        <v>53.3</v>
       </c>
       <c r="S78" t="n">
-        <v>5.8</v>
+        <v>28.7</v>
       </c>
       <c r="X78" t="inlineStr">
         <is>
-          <t>No reportó al MEN</t>
-        </is>
-      </c>
-      <c r="AB78" t="inlineStr">
-        <is>
-          <t>Sin concepto técnico ni reporte del rector</t>
+          <t>Riesgo inminente de colapso</t>
+        </is>
+      </c>
+      <c r="Y78" t="inlineStr">
+        <is>
+          <t>Critico</t>
         </is>
       </c>
       <c r="AC78" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>via principal pavimentada</t>
         </is>
       </c>
       <c r="AD78" t="inlineStr">
@@ -10968,7 +10908,12 @@
       </c>
       <c r="AE78" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 17 m de esa vía.</t>
+          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 37 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AF78" t="inlineStr">
+        <is>
+          <t>Vía a Tienda Nueva</t>
         </is>
       </c>
       <c r="AG78" t="inlineStr">
@@ -10977,10 +10922,10 @@
         </is>
       </c>
       <c r="AH78" t="n">
-        <v>3.528177503</v>
+        <v>3.564564</v>
       </c>
       <c r="AI78" t="n">
-        <v>-76.28814192999999</v>
+        <v>-76.231579</v>
       </c>
     </row>
     <row r="79">
@@ -10995,19 +10940,19 @@
         </is>
       </c>
       <c r="C79" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>sábado</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>6</v>
+      </c>
+      <c r="F79" t="n">
         <v>2</v>
       </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>lunes</t>
-        </is>
-      </c>
-      <c r="E79" t="n">
-        <v>7</v>
-      </c>
-      <c r="F79" t="n">
-        <v>1</v>
-      </c>
       <c r="G79" t="inlineStr">
         <is>
           <t>Palmira</t>
@@ -11015,17 +10960,17 @@
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>ENELIA RIVERA</t>
+          <t>ROSARIO DE FATIMA</t>
         </is>
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA SANTA BARBARA</t>
+          <t>INSTITUCION EDUCATIVA TABLONES</t>
         </is>
       </c>
       <c r="J79" s="3" t="inlineStr">
         <is>
-          <t>176520001957</t>
+          <t>276520000742</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -11035,12 +10980,12 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>CLL 30 CR 40</t>
+          <t>CORREG LA BOLSA</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -11054,57 +10999,57 @@
         </is>
       </c>
       <c r="P79" t="n">
-        <v>6</v>
+        <v>2.14</v>
       </c>
       <c r="Q79" t="n">
-        <v>4.8</v>
+        <v>17.42</v>
       </c>
       <c r="R79" t="n">
-        <v>16.6</v>
+        <v>53.3</v>
       </c>
       <c r="S79" t="n">
-        <v>5.5</v>
+        <v>28.7</v>
       </c>
       <c r="X79" t="inlineStr">
         <is>
-          <t>Afectación menor</t>
+          <t>Colapso parcial</t>
         </is>
       </c>
       <c r="Y79" t="inlineStr">
         <is>
-          <t>Bajo</t>
+          <t>Critico</t>
         </is>
       </c>
       <c r="AC79" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>camino destapado</t>
         </is>
       </c>
       <c r="AD79" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="AE79" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 48 m de esa vía.</t>
+          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 18 m de esa vía.</t>
         </is>
       </c>
       <c r="AF79" t="inlineStr">
         <is>
-          <t>Carrera 41</t>
+          <t>La Bolsa</t>
         </is>
       </c>
       <c r="AG79" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AH79" t="n">
-        <v>3.528369858</v>
+        <v>3.555961</v>
       </c>
       <c r="AI79" t="n">
-        <v>-76.30969955</v>
+        <v>-76.23436599999999</v>
       </c>
     </row>
     <row r="80">
@@ -11130,7 +11075,7 @@
         <v>7</v>
       </c>
       <c r="F80" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -11139,17 +11084,17 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>DOMINGO IRURITA</t>
+          <t>ROSARIO MENESSES</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA DOMINGO IRURITA</t>
+          <t>INSTITUCION EDUCATIVA SAGRADA FAMILIA POTRERILLO</t>
         </is>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>176520002163</t>
+          <t>276520001676</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -11159,12 +11104,12 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>CL 23 33 A 37</t>
+          <t>VDA LOS CUCHOS</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -11178,57 +11123,52 @@
         </is>
       </c>
       <c r="P80" t="n">
-        <v>4.8</v>
+        <v>49.13</v>
       </c>
       <c r="Q80" t="n">
-        <v>5.78</v>
+        <v>33.35</v>
       </c>
       <c r="R80" t="n">
-        <v>16.6</v>
+        <v>110.6</v>
       </c>
       <c r="S80" t="n">
-        <v>5.5</v>
+        <v>52.9</v>
       </c>
       <c r="X80" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
-        </is>
-      </c>
-      <c r="Y80" t="inlineStr">
-        <is>
-          <t>Moderado</t>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB80" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
         </is>
       </c>
       <c r="AC80" t="inlineStr">
         <is>
-          <t>via terciaria</t>
+          <t>camino rural sin categoria</t>
         </is>
       </c>
       <c r="AD80" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="AE80" t="inlineStr">
         <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 35 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AF80" t="inlineStr">
-        <is>
-          <t>Carrera 33A</t>
+          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 37 m de esa vía.</t>
         </is>
       </c>
       <c r="AG80" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AH80" t="n">
-        <v>3.521358245</v>
+        <v>3.550561</v>
       </c>
       <c r="AI80" t="n">
-        <v>-76.30535072000001</v>
+        <v>-76.167422</v>
       </c>
     </row>
     <row r="81">
@@ -11247,14 +11187,14 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>martes</t>
+          <t>lunes</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G81" t="inlineStr">
         <is>
@@ -11263,17 +11203,17 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>JOSE MANUEL GROOT</t>
+          <t>TABLONES</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA HAROLD EDER</t>
+          <t>INSTITUCION EDUCATIVA TABLONES</t>
         </is>
       </c>
       <c r="J81" s="3" t="inlineStr">
         <is>
-          <t>276520002192</t>
+          <t>276520000564</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -11283,12 +11223,12 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>CL 65 31 C 95</t>
+          <t>CORREG TABLONES</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -11302,45 +11242,40 @@
         </is>
       </c>
       <c r="P81" t="n">
-        <v>10.39</v>
+        <v>33.35</v>
       </c>
       <c r="Q81" t="n">
-        <v>8.789999999999999</v>
+        <v>28.1</v>
       </c>
       <c r="R81" t="n">
-        <v>21.8</v>
+        <v>110.6</v>
       </c>
       <c r="S81" t="n">
-        <v>7.6</v>
+        <v>52.9</v>
       </c>
       <c r="X81" t="inlineStr">
         <is>
-          <t>Riesgo inminente de colapso</t>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr">
         <is>
-          <t>Critico</t>
+          <t>Moderado</t>
         </is>
       </c>
       <c r="AC81" t="inlineStr">
         <is>
-          <t>calle de casco urbano</t>
+          <t>camino destapado</t>
         </is>
       </c>
       <c r="AD81" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="AE81" t="inlineStr">
         <is>
-          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 2 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AF81" t="inlineStr">
-        <is>
-          <t>Carrera 32</t>
+          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 21 m de esa vía.</t>
         </is>
       </c>
       <c r="AG81" t="inlineStr">
@@ -11349,10 +11284,10 @@
         </is>
       </c>
       <c r="AH81" t="n">
-        <v>3.556083</v>
+        <v>3.602559</v>
       </c>
       <c r="AI81" t="n">
-        <v>-76.30073299999999</v>
+        <v>-76.20097800000001</v>
       </c>
     </row>
     <row r="82">
@@ -11378,7 +11313,7 @@
         <v>8</v>
       </c>
       <c r="F82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G82" t="inlineStr">
         <is>
@@ -11387,17 +11322,17 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>LICEO FEMENINO</t>
+          <t>LA NEVERA</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DEL PALMAR</t>
+          <t>INSTITUCION EDUCATIVA SAGRADA FAMILIA POTRERILLO</t>
         </is>
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>176520000489</t>
+          <t>276520003032</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -11407,12 +11342,12 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Urbana</t>
+          <t>Rural</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>CR 28 NO 37 81</t>
+          <t>VDA LA NEVERA</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -11426,16 +11361,16 @@
         </is>
       </c>
       <c r="P82" t="n">
-        <v>8.789999999999999</v>
+        <v>88.3</v>
       </c>
       <c r="Q82" t="n">
-        <v>2.66</v>
+        <v>94.04000000000001</v>
       </c>
       <c r="R82" t="n">
-        <v>21.8</v>
+        <v>182.3</v>
       </c>
       <c r="S82" t="n">
-        <v>7.6</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="X82" t="inlineStr">
         <is>
@@ -11449,34 +11384,29 @@
       </c>
       <c r="AC82" t="inlineStr">
         <is>
-          <t>via principal pavimentada</t>
+          <t>camino rural sin categoria</t>
         </is>
       </c>
       <c r="AD82" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="AE82" t="inlineStr">
         <is>
-          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 43 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AF82" t="inlineStr">
-        <is>
-          <t>Carrera 28</t>
+          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 901 m de esa vía.</t>
         </is>
       </c>
       <c r="AG82" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AH82" t="n">
-        <v>3.53438389943</v>
+        <v>3.5386</v>
       </c>
       <c r="AI82" t="n">
-        <v>-76.2982293309</v>
+        <v>-76.1206</v>
       </c>
     </row>
     <row r="83">
@@ -11511,7 +11441,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>CRISTOBAL COLON</t>
+          <t>RITA SABOGAL</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -11521,7 +11451,7 @@
       </c>
       <c r="J83" s="3" t="inlineStr">
         <is>
-          <t>276520001552</t>
+          <t>276520001633</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -11536,7 +11466,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>VDA LA CASCADA</t>
+          <t>VDA TIATINO</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -11550,57 +11480,52 @@
         </is>
       </c>
       <c r="P83" t="n">
-        <v>33.72</v>
+        <v>94.26000000000001</v>
       </c>
       <c r="Q83" t="n">
-        <v>22.95</v>
+        <v>74.64</v>
       </c>
       <c r="R83" t="n">
-        <v>99.40000000000001</v>
+        <v>168.9</v>
       </c>
       <c r="S83" t="n">
-        <v>56.1</v>
+        <v>80.3</v>
       </c>
       <c r="X83" t="inlineStr">
         <is>
-          <t>Riesgo inminente de colapso</t>
-        </is>
-      </c>
-      <c r="Y83" t="inlineStr">
-        <is>
-          <t>Critico</t>
+          <t>No reportó al MEN</t>
+        </is>
+      </c>
+      <c r="AB83" t="inlineStr">
+        <is>
+          <t>Sin concepto técnico ni reporte del rector</t>
         </is>
       </c>
       <c r="AC83" t="inlineStr">
         <is>
-          <t>via principal pavimentada</t>
+          <t>camino rural sin categoria</t>
         </is>
       </c>
       <c r="AD83" t="inlineStr">
         <is>
-          <t>fácil</t>
+          <t>difícil</t>
         </is>
       </c>
       <c r="AE83" t="inlineStr">
         <is>
-          <t>La vía de entrada es via principal pavimentada según OpenStreetMap (clase «secondary»). La sede queda a 37 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AF83" t="inlineStr">
-        <is>
-          <t>Vía a Tienda Nueva</t>
+          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 13 m de esa vía.</t>
         </is>
       </c>
       <c r="AG83" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AH83" t="n">
-        <v>3.564564</v>
+        <v>3.646588</v>
       </c>
       <c r="AI83" t="n">
-        <v>-76.231579</v>
+        <v>-76.06974599999999</v>
       </c>
     </row>
     <row r="84">
@@ -11619,14 +11544,14 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>miércoles</t>
+          <t>jueves</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F84" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -11635,17 +11560,17 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>MARCO FIDEL SUAREZ</t>
+          <t>ALFONSO LOPEZ PUMAREJO</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA TABLONES</t>
+          <t>INSTITUCION EDUCATIVA ALFONSO LOPEZ PUMAREJO</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>276520001684</t>
+          <t>176520002091</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -11655,12 +11580,12 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>VDA LA ESPERANZA</t>
+          <t>KR 16 32 02</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -11670,24 +11595,24 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="P84" t="n">
-        <v>22.95</v>
+        <v>7.29</v>
       </c>
       <c r="Q84" t="n">
-        <v>42.74</v>
+        <v>33.77</v>
       </c>
       <c r="R84" t="n">
-        <v>99.40000000000001</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="S84" t="n">
-        <v>56.1</v>
+        <v>48.8</v>
       </c>
       <c r="X84" t="inlineStr">
         <is>
-          <t>No está en la capa del MEN</t>
+          <t>No reportó al MEN</t>
         </is>
       </c>
       <c r="AB84" t="inlineStr">
@@ -11697,7 +11622,7 @@
       </c>
       <c r="AC84" t="inlineStr">
         <is>
-          <t>via terciaria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="AD84" t="inlineStr">
@@ -11707,7 +11632,7 @@
       </c>
       <c r="AE84" t="inlineStr">
         <is>
-          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 9 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «service»). La sede queda a 17 m de esa vía.</t>
         </is>
       </c>
       <c r="AG84" t="inlineStr">
@@ -11716,10 +11641,10 @@
         </is>
       </c>
       <c r="AH84" t="n">
-        <v>3.610511</v>
+        <v>3.528177503</v>
       </c>
       <c r="AI84" t="n">
-        <v>-76.155193</v>
+        <v>-76.28814192999999</v>
       </c>
     </row>
     <row r="85">
@@ -11745,7 +11670,7 @@
         <v>10</v>
       </c>
       <c r="F85" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G85" t="inlineStr">
         <is>
@@ -11754,17 +11679,17 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>MARIA DOMINGUEZ</t>
+          <t>SANTO TOMAS DE AQUINO</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA SAGRADA FAMILIA POTRERILLO</t>
+          <t>INSTITUCION EDUCATIVA FRANCISCO MIRANDA</t>
         </is>
       </c>
       <c r="J85" s="3" t="inlineStr">
         <is>
-          <t>276520001625</t>
+          <t>276520000548</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -11779,7 +11704,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>VDA LA MARIA</t>
+          <t>VDA MESON</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -11789,24 +11714,24 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="P85" t="n">
-        <v>58.29</v>
+        <v>33.77</v>
       </c>
       <c r="Q85" t="n">
-        <v>68.20999999999999</v>
+        <v>52.56</v>
       </c>
       <c r="R85" t="n">
-        <v>126.5</v>
+        <v>93.59999999999999</v>
       </c>
       <c r="S85" t="n">
-        <v>49.7</v>
+        <v>48.8</v>
       </c>
       <c r="X85" t="inlineStr">
         <is>
-          <t>No está en la capa del MEN</t>
+          <t>No reportó al MEN</t>
         </is>
       </c>
       <c r="AB85" t="inlineStr">
@@ -11816,34 +11741,29 @@
       </c>
       <c r="AC85" t="inlineStr">
         <is>
-          <t>camino destapado</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="AD85" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="AE85" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 16 m de esa vía.</t>
-        </is>
-      </c>
-      <c r="AF85" t="inlineStr">
-        <is>
-          <t>Via Tenjo - Mariala Alta</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 12 m de esa vía.</t>
         </is>
       </c>
       <c r="AG85" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AH85" t="n">
-        <v>3.510825276</v>
+        <v>3.497136</v>
       </c>
       <c r="AI85" t="n">
-        <v>-76.14317477</v>
+        <v>-76.190214</v>
       </c>
     </row>
     <row r="86">
@@ -11873,60 +11793,75 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>BID (43)</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>TABLONES</t>
+          <t>ALFONSO LOPEZ PUMAREJO</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA TABLONES</t>
+          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DE LA CANDELARIA</t>
         </is>
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>276520000564</t>
+          <t>176130000330</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>CANDELARIA</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>CORREG TABLONES</t>
+          <t>CL 7 9 11</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="P86" t="n">
-        <v>38.78</v>
+        <v>0.23</v>
       </c>
       <c r="Q86" t="n">
-        <v>25.67</v>
+        <v>1.88</v>
       </c>
       <c r="R86" t="n">
-        <v>117.8</v>
+        <v>2.1</v>
       </c>
       <c r="S86" t="n">
-        <v>61</v>
+        <v>0.6</v>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>PATOLOGIA ESTRUCTURAL</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>No habitable</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>aprobado por la mesa</t>
+        </is>
       </c>
       <c r="X86" t="inlineStr">
         <is>
@@ -11938,19 +11873,29 @@
           <t>Moderado</t>
         </is>
       </c>
+      <c r="Z86" t="inlineStr">
+        <is>
+          <t>Afectación parcial</t>
+        </is>
+      </c>
       <c r="AC86" t="inlineStr">
         <is>
-          <t>camino destapado</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="AD86" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="AE86" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «track», la clase de los caminos de uso agrícola o forestal. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 21 m de esa vía.</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 2 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AF86" t="inlineStr">
+        <is>
+          <t>Calle 7</t>
         </is>
       </c>
       <c r="AG86" t="inlineStr">
@@ -11959,10 +11904,10 @@
         </is>
       </c>
       <c r="AH86" t="n">
-        <v>3.602559</v>
+        <v>3.407489</v>
       </c>
       <c r="AI86" t="n">
-        <v>-76.20097800000001</v>
+        <v>-76.34917799999999</v>
       </c>
     </row>
     <row r="87">
@@ -11981,107 +11926,132 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>viernes</t>
+          <t>sábado</t>
         </is>
       </c>
       <c r="E87" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>BID (43)</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>ROSARIO MENESSES</t>
+          <t>SAGRADA FAMILIA</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA SAGRADA FAMILIA POTRERILLO</t>
+          <t>INSTITUCION EDUCATIVA NUESTRA SEÑORA DE LA CANDELARIA</t>
         </is>
       </c>
       <c r="J87" s="3" t="inlineStr">
         <is>
-          <t>276520001676</t>
+          <t>176130000356</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>CANDELARIA</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>VDA LOS CUCHOS</t>
+          <t>CL 7 8 42</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="P87" t="n">
-        <v>25.67</v>
+        <v>0.44</v>
       </c>
       <c r="Q87" t="n">
-        <v>53.34</v>
+        <v>1.68</v>
       </c>
       <c r="R87" t="n">
-        <v>117.8</v>
+        <v>2.1</v>
       </c>
       <c r="S87" t="n">
-        <v>61</v>
+        <v>0.6</v>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>PATOLOGIA ESTRUCTURAL</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>No habitable</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>aprobado por la mesa</t>
+        </is>
       </c>
       <c r="X87" t="inlineStr">
         <is>
-          <t>No reportó al MEN</t>
-        </is>
-      </c>
-      <c r="AB87" t="inlineStr">
-        <is>
-          <t>Sin concepto técnico ni reporte del rector</t>
+          <t>Afectación parcial</t>
+        </is>
+      </c>
+      <c r="Y87" t="inlineStr">
+        <is>
+          <t>Moderado</t>
+        </is>
+      </c>
+      <c r="Z87" t="inlineStr">
+        <is>
+          <t>Afectación parcial</t>
         </is>
       </c>
       <c r="AC87" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>via terciaria</t>
         </is>
       </c>
       <c r="AD87" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="AE87" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 1330 m de esa vía.</t>
+          <t>La vía de entrada es via terciaria según OpenStreetMap (clase «tertiary»). La sede queda a 33 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AF87" t="inlineStr">
+        <is>
+          <t>Calle 7</t>
         </is>
       </c>
       <c r="AG87" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AH87" t="n">
-        <v>3.582859967</v>
+        <v>3.40761667</v>
       </c>
       <c r="AI87" t="n">
-        <v>-76.15750609</v>
+        <v>-76.34858894</v>
       </c>
     </row>
     <row r="88">
@@ -12096,111 +12066,121 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>sábado</t>
+          <t>lunes</t>
         </is>
       </c>
       <c r="E88" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F88" t="n">
         <v>1</v>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>BID (43)</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>LA NEVERA</t>
+          <t>SAGRADO CORAZON DE JESUS</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA SAGRADA FAMILIA POTRERILLO</t>
+          <t>INSTITUCION EDUCATIVA ABSALON TORRES CAMACHO</t>
         </is>
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>276520003032</t>
+          <t>176275000125</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>FLORIDA</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>Rural</t>
+          <t>Urbana</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>VDA LA NEVERA</t>
+          <t>CR 21 NO 9-89</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="P88" t="n">
-        <v>99.38</v>
+        <v>27.65</v>
       </c>
       <c r="Q88" t="n">
-        <v>104.79</v>
+        <v>28.95</v>
       </c>
       <c r="R88" t="n">
-        <v>204.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="S88" t="n">
-        <v>81.09999999999999</v>
+        <v>44</v>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>PATOLOGIA ESTRUCTURAL</t>
+        </is>
       </c>
       <c r="X88" t="inlineStr">
         <is>
-          <t>Afectación parcial</t>
+          <t>Afectación menor</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Bajo</t>
         </is>
       </c>
       <c r="AC88" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="AD88" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="AE88" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 272 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 23 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AF88" t="inlineStr">
+        <is>
+          <t>Calle 10</t>
         </is>
       </c>
       <c r="AG88" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AH88" t="n">
-        <v>3.545813</v>
+        <v>3.32644406118</v>
       </c>
       <c r="AI88" t="n">
-        <v>-76.113687</v>
+        <v>-76.23742270629999</v>
       </c>
     </row>
     <row r="89">
@@ -12226,31 +12206,31 @@
         <v>13</v>
       </c>
       <c r="F89" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>BID (43)</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>RITA SABOGAL</t>
+          <t>JOSE EUSEBIO CARO</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>INSTITUCION EDUCATIVA TABLONES</t>
+          <t>INSTITUCION EDUCATIVA INMACULADA CONCEPCION</t>
         </is>
       </c>
       <c r="J89" s="3" t="inlineStr">
         <is>
-          <t>276520001633</t>
+          <t>276130000288</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>CANDELARIA</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -12260,66 +12240,91 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>VDA TIATINO</t>
+          <t>CR 12 NO 10-81</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="P89" t="n">
-        <v>98.42</v>
+        <v>28.95</v>
       </c>
       <c r="Q89" t="n">
-        <v>79.44</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="R89" t="n">
-        <v>177.9</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="S89" t="n">
-        <v>83.90000000000001</v>
+        <v>44</v>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>PATOLOGIA ESTRUCTURAL</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>No habitable</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>aprobado por la mesa</t>
+        </is>
       </c>
       <c r="X89" t="inlineStr">
         <is>
-          <t>No reportó al MEN</t>
-        </is>
-      </c>
-      <c r="AB89" t="inlineStr">
-        <is>
-          <t>Sin concepto técnico ni reporte del rector</t>
+          <t>Afectación menor</t>
+        </is>
+      </c>
+      <c r="Y89" t="inlineStr">
+        <is>
+          <t>Bajo</t>
+        </is>
+      </c>
+      <c r="Z89" t="inlineStr">
+        <is>
+          <t>Afectación menor</t>
         </is>
       </c>
       <c r="AC89" t="inlineStr">
         <is>
-          <t>camino rural sin categoria</t>
+          <t>calle de casco urbano</t>
         </is>
       </c>
       <c r="AD89" t="inlineStr">
         <is>
-          <t>difícil</t>
+          <t>fácil</t>
         </is>
       </c>
       <c r="AE89" t="inlineStr">
         <is>
-          <t>OpenStreetMap la marca como «unclassified», una vía menor por debajo de las terciarias. La clase no dice si está pavimentada; conviene confirmar el estado antes de salir. La sede queda a 352 m de esa vía.</t>
+          <t>La vía de entrada es calle de casco urbano según OpenStreetMap (clase «residential»). La sede queda a 1 m de esa vía.</t>
+        </is>
+      </c>
+      <c r="AF89" t="inlineStr">
+        <is>
+          <t>CALLEJON FLORO MERCADO CRUCE VIA 13025VL04-2E</t>
         </is>
       </c>
       <c r="AG89" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="AH89" t="n">
-        <v>3.641394707</v>
+        <v>3.39537597879</v>
       </c>
       <c r="AI89" t="n">
-        <v>-76.05537963</v>
+        <v>-76.3859481842</v>
       </c>
     </row>
     <row r="90">
@@ -12384,7 +12389,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -12393,16 +12398,16 @@
         </is>
       </c>
       <c r="P90" t="n">
-        <v>29.19</v>
+        <v>36.99</v>
       </c>
       <c r="Q90" t="n">
         <v>11.21</v>
       </c>
       <c r="R90" t="n">
-        <v>77.59999999999999</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="S90" t="n">
-        <v>52.2</v>
+        <v>60.7</v>
       </c>
       <c r="X90" t="inlineStr">
         <is>
@@ -12503,7 +12508,7 @@
       </c>
       <c r="N91" t="inlineStr">
         <is>
-          <t>Palmira</t>
+          <t>Candelaria</t>
         </is>
       </c>
       <c r="O91" t="inlineStr">
@@ -12518,10 +12523,10 @@
         <v>37.19</v>
       </c>
       <c r="R91" t="n">
-        <v>77.59999999999999</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="S91" t="n">
-        <v>52.2</v>
+        <v>60.7</v>
       </c>
       <c r="X91" t="inlineStr">
         <is>
@@ -12599,7 +12604,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-02</t>
         </is>
       </c>
     </row>
@@ -12800,10 +12805,10 @@
         <v>24</v>
       </c>
       <c r="D14" t="n">
-        <v>18.9</v>
+        <v>15.1</v>
       </c>
       <c r="E14" t="n">
-        <v>572</v>
+        <v>461</v>
       </c>
       <c r="F14" t="n">
         <v>13</v>

</xml_diff>